<commit_message>
Update steps - 1st to 15th
</commit_message>
<xml_diff>
--- a/data/steps.xlsx
+++ b/data/steps.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -59,6 +59,21 @@
   </si>
   <si>
     <t>10-09-26</t>
+  </si>
+  <si>
+    <t>11-09-26</t>
+  </si>
+  <si>
+    <t>12-09-26</t>
+  </si>
+  <si>
+    <t>13-09-26</t>
+  </si>
+  <si>
+    <t>14-09-26</t>
+  </si>
+  <si>
+    <t>15-09-26</t>
   </si>
 </sst>
 </file>
@@ -542,19 +557,104 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2"/>
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="3">
+        <v>13334.0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>7740.0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>12598.0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>6372.0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>3729.0</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2"/>
+      <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3">
+        <v>6200.0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>5499.0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>10361.0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>15260.0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1749.0</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2"/>
+      <c r="A14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="3">
+        <v>18255.0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>5433.0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>13214.0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>9392.0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>3786.0</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2"/>
+      <c r="A15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="3">
+        <v>5474.0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>5517.0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>11949.0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>10789.0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>7486.0</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2"/>
+      <c r="A16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="3">
+        <v>12457.0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4807.0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>13825.0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>15234.0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>3071.0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2"/>

</xml_diff>

<commit_message>
Update Count : 1st - 20th Sept
</commit_message>
<xml_diff>
--- a/data/steps.xlsx
+++ b/data/steps.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -74,6 +74,21 @@
   </si>
   <si>
     <t>15-09-26</t>
+  </si>
+  <si>
+    <t>16-09-26</t>
+  </si>
+  <si>
+    <t>17-09-26</t>
+  </si>
+  <si>
+    <t>18-09-26</t>
+  </si>
+  <si>
+    <t>19-09-26</t>
+  </si>
+  <si>
+    <t>20-09-26</t>
   </si>
 </sst>
 </file>
@@ -657,19 +672,104 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2"/>
+      <c r="A17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3">
+        <v>8426.0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>5449.0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>11430.0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>15199.0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>4693.0</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2"/>
+      <c r="A18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="3">
+        <v>7626.0</v>
+      </c>
+      <c r="C18" s="3">
+        <v>5248.0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>13647.0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>11036.0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>7541.0</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2"/>
+      <c r="A19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="3">
+        <v>9161.0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>8392.0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>11488.0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>14470.0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>5072.0</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2"/>
+      <c r="A20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="3">
+        <v>2662.0</v>
+      </c>
+      <c r="C20" s="3">
+        <v>8876.0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>17279.0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>9619.0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>2885.0</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2"/>
+      <c r="A21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="3">
+        <v>5977.0</v>
+      </c>
+      <c r="C21" s="3">
+        <v>10104.0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>16074.0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>7009.0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>2415.0</v>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2"/>
@@ -1295,9 +1395,7 @@
     <row r="229" ht="15.75" customHeight="1">
       <c r="A229" s="2"/>
     </row>
-    <row r="230" ht="15.75" customHeight="1">
-      <c r="A230" s="2"/>
-    </row>
+    <row r="230" ht="15.75" customHeight="1"/>
     <row r="231" ht="15.75" customHeight="1"/>
     <row r="232" ht="15.75" customHeight="1"/>
     <row r="233" ht="15.75" customHeight="1"/>
@@ -2067,7 +2165,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>